<commit_message>
remove text in column P (after renaming Titel -> ColP)
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu.xlsx
+++ b/tests/testthat/excel/mapping_neu.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D9FA419-E7F0-437C-9092-82E1700B70F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{328A15E7-A9F5-4382-8626-2F98CBDA4309}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15525" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15525" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Config" sheetId="1" r:id="rId1"/>
@@ -1729,13 +1729,13 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>6</xdr:col>
-          <xdr:colOff>800100</xdr:colOff>
+          <xdr:colOff>352425</xdr:colOff>
           <xdr:row>0</xdr:row>
           <xdr:rowOff>47625</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>6</xdr:col>
-          <xdr:colOff>2324100</xdr:colOff>
+          <xdr:colOff>1876425</xdr:colOff>
           <xdr:row>0</xdr:row>
           <xdr:rowOff>228600</xdr:rowOff>
         </xdr:to>
@@ -14569,10 +14569,7 @@
       <c r="M3" s="25"/>
       <c r="N3" s="25"/>
       <c r="O3" s="25"/>
-      <c r="P3" s="31" t="str">
-        <f t="shared" ref="P3:P18" si="0">IF(B3&lt;&gt;"",A3&amp;"}"&amp;B3,"")</f>
-        <v/>
-      </c>
+      <c r="P3" s="31"/>
       <c r="Q3" s="25"/>
       <c r="R3" s="25"/>
       <c r="S3" s="25"/>
@@ -14611,10 +14608,7 @@
       <c r="M4" s="25"/>
       <c r="N4" s="25"/>
       <c r="O4" s="25"/>
-      <c r="P4" s="31" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
+      <c r="P4" s="31"/>
       <c r="Q4" s="25"/>
       <c r="R4" s="25"/>
       <c r="S4" s="25"/>
@@ -14663,10 +14657,7 @@
       <c r="M5" s="31"/>
       <c r="N5" s="31"/>
       <c r="O5" s="25"/>
-      <c r="P5" s="31" t="str">
-        <f t="shared" si="0"/>
-        <v>}Region</v>
-      </c>
+      <c r="P5" s="31"/>
       <c r="Q5" s="31"/>
       <c r="R5" s="25"/>
       <c r="S5" s="25"/>
@@ -14720,10 +14711,7 @@
       <c r="M6" s="31"/>
       <c r="N6" s="31"/>
       <c r="O6" s="25"/>
-      <c r="P6" s="31" t="str">
-        <f t="shared" si="0"/>
-        <v>Q1}1. Wie viele Mitarbeiter beschäftigt Ihr Unternehmen?</v>
-      </c>
+      <c r="P6" s="31"/>
       <c r="Q6" s="31"/>
       <c r="R6" s="31"/>
       <c r="S6" s="31"/>
@@ -14752,7 +14740,7 @@
     </row>
     <row r="7" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A7" s="30" t="str">
-        <f t="shared" ref="A7:A18" si="1">"Q"&amp;LEFT(B7,FIND(".",B7)-1)</f>
+        <f t="shared" ref="A7:A18" si="0">"Q"&amp;LEFT(B7,FIND(".",B7)-1)</f>
         <v>Q2</v>
       </c>
       <c r="B7" s="30" t="s">
@@ -14777,10 +14765,7 @@
       <c r="M7" s="31"/>
       <c r="N7" s="31"/>
       <c r="O7" s="25"/>
-      <c r="P7" s="31" t="str">
-        <f t="shared" si="0"/>
-        <v>Q2}2. Welche Art von Studien führen Sie mit dem Tabellenbandtool durch?' 'DC#SELVALLAB</v>
-      </c>
+      <c r="P7" s="31"/>
       <c r="Q7" s="31"/>
       <c r="R7" s="31"/>
       <c r="S7" s="31" t="s">
@@ -14813,7 +14798,7 @@
     </row>
     <row r="8" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A8" s="30" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>Q3</v>
       </c>
       <c r="B8" s="30" t="s">
@@ -14840,10 +14825,7 @@
         <v>259</v>
       </c>
       <c r="O8" s="25"/>
-      <c r="P8" s="31" t="str">
-        <f t="shared" si="0"/>
-        <v>Q3}3. Wie verteilten sich die Studien prozentual auf die einzelnen Arten?</v>
-      </c>
+      <c r="P8" s="31"/>
       <c r="Q8" s="31"/>
       <c r="R8" s="31"/>
       <c r="S8" s="31"/>
@@ -14872,7 +14854,7 @@
     </row>
     <row r="9" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A9" s="30" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>Q4</v>
       </c>
       <c r="B9" s="30" t="s">
@@ -14903,10 +14885,7 @@
         <v>263</v>
       </c>
       <c r="O9" s="25"/>
-      <c r="P9" s="31" t="str">
-        <f t="shared" si="0"/>
-        <v xml:space="preserve">Q4}4. Wie häufig haben Sie einen Tabellenband in den letzten 12 Monaten erstellen lassen? </v>
-      </c>
+      <c r="P9" s="31"/>
       <c r="Q9" s="31"/>
       <c r="R9" s="31"/>
       <c r="S9" s="31"/>
@@ -14935,7 +14914,7 @@
     </row>
     <row r="10" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A10" s="30" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>Q5</v>
       </c>
       <c r="B10" s="30" t="s">
@@ -14960,10 +14939,7 @@
       <c r="M10" s="31"/>
       <c r="N10" s="31"/>
       <c r="O10" s="25"/>
-      <c r="P10" s="31" t="str">
-        <f t="shared" si="0"/>
-        <v>Q5}5. Was lief besonders gut in den Projekten?</v>
-      </c>
+      <c r="P10" s="31"/>
       <c r="Q10" s="31" t="s">
         <v>294</v>
       </c>
@@ -14996,7 +14972,7 @@
     </row>
     <row r="11" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A11" s="30" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>Q5</v>
       </c>
       <c r="B11" s="30" t="s">
@@ -15027,10 +15003,7 @@
       <c r="M11" s="31"/>
       <c r="N11" s="31"/>
       <c r="O11" s="25"/>
-      <c r="P11" s="31" t="str">
-        <f t="shared" si="0"/>
-        <v>Q5}5. Was lief besonders gut in den Projekten?</v>
-      </c>
+      <c r="P11" s="31"/>
       <c r="Q11" s="31" t="s">
         <v>295</v>
       </c>
@@ -15061,7 +15034,7 @@
     </row>
     <row r="12" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A12" s="30" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>Q5</v>
       </c>
       <c r="B12" s="30" t="s">
@@ -15092,10 +15065,7 @@
       <c r="M12" s="31"/>
       <c r="N12" s="31"/>
       <c r="O12" s="25"/>
-      <c r="P12" s="31" t="str">
-        <f t="shared" si="0"/>
-        <v>Q5}5. Was lief besonders gut in den Projekten?</v>
-      </c>
+      <c r="P12" s="31"/>
       <c r="Q12" s="31"/>
       <c r="R12" s="31"/>
       <c r="S12" s="31"/>
@@ -15146,10 +15116,7 @@
       <c r="M13" s="31"/>
       <c r="N13" s="31"/>
       <c r="O13" s="25"/>
-      <c r="P13" s="31" t="str">
-        <f t="shared" si="0"/>
-        <v>}Abgefragte Studienarten</v>
-      </c>
+      <c r="P13" s="31"/>
       <c r="Q13" s="31" t="s">
         <v>296</v>
       </c>
@@ -15182,7 +15149,7 @@
     </row>
     <row r="14" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A14" s="30" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>Q6</v>
       </c>
       <c r="B14" s="30" t="s">
@@ -15213,10 +15180,7 @@
         <v>259</v>
       </c>
       <c r="O14" s="25"/>
-      <c r="P14" s="31" t="str">
-        <f t="shared" si="0"/>
-        <v>Q6}6. Ich nenne Ihnen gleich einige generelle Merkmale, die bei quantitativen Forschungsprojekten eine Rolle spielen. Bitte stufen Sie die Wichtigkeit ein.</v>
-      </c>
+      <c r="P14" s="31"/>
       <c r="Q14" s="31"/>
       <c r="R14" s="31"/>
       <c r="S14" s="31"/>
@@ -15249,7 +15213,7 @@
     </row>
     <row r="15" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A15" s="30" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>Q7</v>
       </c>
       <c r="B15" s="30" t="s">
@@ -15280,10 +15244,7 @@
         <v>259</v>
       </c>
       <c r="O15" s="25"/>
-      <c r="P15" s="31" t="str">
-        <f t="shared" si="0"/>
-        <v>Q7}7. Für die abgefragten Studienarten: Wie zufrieden sind Sie mit dem Tabellenbandtool bezüglich der eben abgefragten Merkmale?' 'DC#SELVALLAB</v>
-      </c>
+      <c r="P15" s="31"/>
       <c r="Q15" s="31"/>
       <c r="R15" s="31"/>
       <c r="S15" s="31" t="s">
@@ -15318,7 +15279,7 @@
     </row>
     <row r="16" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A16" s="30" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>Q8</v>
       </c>
       <c r="B16" s="30" t="s">
@@ -15349,10 +15310,7 @@
         <v>259</v>
       </c>
       <c r="O16" s="25"/>
-      <c r="P16" s="31" t="str">
-        <f t="shared" si="0"/>
-        <v>Q8}8. Wie zufrieden sind Sie mit dem Tabellenbandtool insgesamt?' 'DC#SELVALLAB</v>
-      </c>
+      <c r="P16" s="31"/>
       <c r="Q16" s="31"/>
       <c r="R16" s="31"/>
       <c r="S16" s="31" t="s">
@@ -15385,7 +15343,7 @@
     </row>
     <row r="17" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A17" s="30" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>Q9</v>
       </c>
       <c r="B17" s="30" t="s">
@@ -15414,10 +15372,7 @@
       <c r="M17" s="31"/>
       <c r="N17" s="31"/>
       <c r="O17" s="25"/>
-      <c r="P17" s="31" t="str">
-        <f t="shared" si="0"/>
-        <v>Q9}9. Würden Sie das Tabellenbandtool weiterempfehlen?' 'DC#SELVALLAB</v>
-      </c>
+      <c r="P17" s="31"/>
       <c r="Q17" s="31"/>
       <c r="R17" s="31"/>
       <c r="S17" s="31" t="s">
@@ -15450,7 +15405,7 @@
     </row>
     <row r="18" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A18" s="30" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>Q10</v>
       </c>
       <c r="B18" s="30" t="s">
@@ -15479,10 +15434,7 @@
         <v>263</v>
       </c>
       <c r="O18" s="25"/>
-      <c r="P18" s="31" t="str">
-        <f t="shared" si="0"/>
-        <v>Q10}10. Dürfte ich Sie noch nach Ihrem Alter fragen?</v>
-      </c>
+      <c r="P18" s="31"/>
       <c r="Q18" s="31"/>
       <c r="R18" s="31"/>
       <c r="S18" s="31"/>
@@ -41287,13 +41239,13 @@
                 <anchor moveWithCells="1">
                   <from>
                     <xdr:col>6</xdr:col>
-                    <xdr:colOff>800100</xdr:colOff>
+                    <xdr:colOff>352425</xdr:colOff>
                     <xdr:row>0</xdr:row>
                     <xdr:rowOff>47625</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>6</xdr:col>
-                    <xdr:colOff>2324100</xdr:colOff>
+                    <xdr:colOff>1876425</xdr:colOff>
                     <xdr:row>0</xdr:row>
                     <xdr:rowOff>228600</xdr:rowOff>
                   </to>

</xml_diff>